<commit_message>
Ran some sweeps with existing molecules
</commit_message>
<xml_diff>
--- a/pureComponents.xlsx
+++ b/pureComponents.xlsx
@@ -8,14 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\aglotov\Eutectics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7598054-EC05-4CB3-8655-7F6B88E25ABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F0BF7A6-8C06-433A-9BB7-F631EB1FA858}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{22E7D031-F429-4E0A-8A8B-4D129F5BB641}"/>
+    <workbookView xWindow="-24840" yWindow="945" windowWidth="21600" windowHeight="14715" xr2:uid="{22E7D031-F429-4E0A-8A8B-4D129F5BB641}"/>
   </bookViews>
   <sheets>
     <sheet name="CATALOG" sheetId="1" r:id="rId1"/>
     <sheet name="Input" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CATALOG!$A$1:$F$1</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -45,7 +48,201 @@
     <author>Alexander Glotov</author>
   </authors>
   <commentList>
-    <comment ref="F2" authorId="0" shapeId="0" xr:uid="{E5BF108A-0EA7-4AC6-92BA-13EC6989AEC0}">
+    <comment ref="D2" authorId="0" shapeId="0" xr:uid="{B7D4224E-A493-447D-84BA-7DDEFFF3C9D8}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+https://pubchem.ncbi.nlm.nih.gov/compound/Water#section=Melting-Point</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E2" authorId="0" shapeId="0" xr:uid="{5995BC99-B557-4A15-B6FB-81F561DA6AD0}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+https://www.engineeringtoolbox.com/water-thermal-properties-d_162.html</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F2" authorId="0" shapeId="0" xr:uid="{783F21FA-4AD3-468F-B910-64A10EB1842D}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://atct.anl.gov/Thermochemical%20Data/version%201.220/species/?species_number=24</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{2C99D34F-09BE-451B-8192-07DB24810E50}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Ashlee</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E3" authorId="0" shapeId="0" xr:uid="{36D0DEA9-FF41-4A3D-B02A-6E8572488186}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Ashlee</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F3" authorId="0" shapeId="0" xr:uid="{380BD958-450B-4177-80CD-D9786D489AA7}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://atct.anl.gov/Thermochemical%20Data/version%201.220/species/?species_number=1912</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D4" authorId="0" shapeId="0" xr:uid="{49F68355-A445-4BAF-90F2-E3C2E9145A46}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Ashlee</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E4" authorId="0" shapeId="0" xr:uid="{ADF150B1-E417-45FE-81D2-E8DAE9F836DF}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Ashlee</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F4" authorId="0" shapeId="0" xr:uid="{E5BF108A-0EA7-4AC6-92BA-13EC6989AEC0}">
       <text>
         <r>
           <rPr>
@@ -70,7 +267,80 @@
         </r>
       </text>
     </comment>
-    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{4248127E-F186-424E-9304-4093375A6B0B}">
+    <comment ref="D5" authorId="0" shapeId="0" xr:uid="{787C61F0-F01E-4D84-8CAA-AAF894740532}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Hilgeman, Mouroux, Mok, Holan</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E5" authorId="0" shapeId="0" xr:uid="{B609F4F6-1D6F-4E43-899A-039D6BA4839B}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Hilgeman, Mouroux, Mok, Holan</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F5" authorId="0" shapeId="0" xr:uid="{4457B27D-9D44-49EE-9499-EE2A8F5DB1FF}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C288324&amp;Units=SI&amp;Mask=2#Thermo-Condensed</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D6" authorId="0" shapeId="0" xr:uid="{4248127E-F186-424E-9304-4093375A6B0B}">
       <text>
         <r>
           <rPr>
@@ -95,7 +365,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E3" authorId="0" shapeId="0" xr:uid="{AEBB7345-F0F7-4DD9-B32E-D9F056EBEF40}">
+    <comment ref="E6" authorId="0" shapeId="0" xr:uid="{AEBB7345-F0F7-4DD9-B32E-D9F056EBEF40}">
       <text>
         <r>
           <rPr>
@@ -120,7 +390,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F3" authorId="0" shapeId="0" xr:uid="{5106F13A-279A-4601-92D6-B2E92F9DD06C}">
+    <comment ref="F6" authorId="0" shapeId="0" xr:uid="{5106F13A-279A-4601-92D6-B2E92F9DD06C}">
       <text>
         <r>
           <rPr>
@@ -142,6 +412,351 @@
           <t xml:space="preserve">
 Source(s):
 1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C141435&amp;Units=SI&amp;Mask=2#Thermo-Condensed</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D7" authorId="0" shapeId="0" xr:uid="{74CA7090-F16F-4E81-9C1D-4C76B0CA001F}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://advanced.onlinelibrary.wiley.com/doi/10.1002/adma.202502566</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D8" authorId="0" shapeId="0" xr:uid="{1E1D85AE-73C9-4EE5-9B10-D99F6D60BD07}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+https://webbook.nist.gov/cgi/cbook.cgi?ID=C111966&amp;Mask=4#Thermo-Phase</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E8" authorId="0" shapeId="0" xr:uid="{EB6033F4-CA7E-49DB-BB17-C34560971AF5}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+https://webbook.nist.gov/cgi/cbook.cgi?ID=C111966&amp;Mask=4#Thermo-Phase</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F8" authorId="0" shapeId="0" xr:uid="{525F711F-3C09-481A-85BF-92F18353722F}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+https://webbook.nist.gov/cgi/cbook.cgi?ID=C111966&amp;Mask=2#Thermo-Condensed</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D9" authorId="0" shapeId="0" xr:uid="{2CF6CDD1-F5E1-43E8-A19E-28BAAD5C627C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+https://webbook.nist.gov/cgi/cbook.cgi?ID=C56815&amp;Units=SI&amp;Mask=4#Thermo-Phase</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E9" authorId="0" shapeId="0" xr:uid="{67560CD9-4B42-4009-8FEE-B7B0E0D24E47}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+https://webbook.nist.gov/cgi/cbook.cgi?ID=C56815&amp;Units=SI&amp;Mask=4#Thermo-Phase</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F9" authorId="0" shapeId="0" xr:uid="{5E82BDD6-5DA8-4D10-AA85-ECD6AB017319}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+https://webbook.nist.gov/cgi/cbook.cgi?ID=C56815&amp;Units=SI&amp;Mask=2#Thermo-Condensed</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D10" authorId="0" shapeId="0" xr:uid="{471E01A8-C311-4AC7-AEC5-5D6B6CAAD97B}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C107153&amp;Mask=1E9F#Thermo-Condensed</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E10" authorId="0" shapeId="0" xr:uid="{CBC558AB-017C-4385-AA76-E249D19B2033}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C107153&amp;Mask=1E9F#Thermo-Condensed</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F10" authorId="0" shapeId="0" xr:uid="{AB8D56E7-0CD8-4253-A680-DB2E9B7966F8}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C107153&amp;Mask=1E9F#Thermo-Condensed</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D11" authorId="0" shapeId="0" xr:uid="{B68F36C1-4BA4-48F1-99E3-8AD353A1321A}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://advanced.onlinelibrary.wiley.com/doi/10.1002/adma.202502566</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F11" authorId="0" shapeId="0" xr:uid="{BADEE219-B2DB-4696-8CD3-185AC97E6E32}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://www.sciencedirect.com/science/article/abs/pii/S0040603115003354
+2)https://www.sciencedirect.com/science/article/pii/S0016236125036129</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D12" authorId="0" shapeId="0" xr:uid="{63C390B0-F0DD-4E22-8006-4770ED582EEB}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://matweb.com/search/datasheet.aspx?MatGUID=3118b2052ace4835a6d73687613def66&amp;ckck=1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F12" authorId="0" shapeId="0" xr:uid="{E1A1E0C1-3AE1-4CDA-A225-D95E0807710C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://matweb.com/search/datasheet.aspx?MatGUID=3118b2052ace4835a6d73687613def66&amp;ckck=1</t>
         </r>
       </text>
     </comment>
@@ -155,7 +770,351 @@
     <author>Alexander Glotov</author>
   </authors>
   <commentList>
-    <comment ref="F2" authorId="0" shapeId="0" xr:uid="{9A32D99D-8711-4F0B-8645-2CCDB24EED87}">
+    <comment ref="D2" authorId="0" shapeId="0" xr:uid="{5501DECC-CA51-4608-A2A9-124DF8574F9C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Ashlee</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E2" authorId="0" shapeId="0" xr:uid="{366F9C8A-C349-48E6-8883-C6E40BE5B81F}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Ashlee</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F2" authorId="0" shapeId="0" xr:uid="{F3DAE571-D049-4F99-B2BB-AD33D024F8CA}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://atct.anl.gov/Thermochemical%20Data/version%201.220/species/?species_number=1912</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{FC2E5BC0-6FB5-46E6-A96C-B5A571D6D42E}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C107153&amp;Mask=1E9F#Thermo-Condensed</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E3" authorId="0" shapeId="0" xr:uid="{97513E38-6E68-43E5-A94C-6F8C909B7BCE}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C107153&amp;Mask=1E9F#Thermo-Condensed</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F3" authorId="0" shapeId="0" xr:uid="{1DBE5D3C-786F-4099-B286-532040D0D3AF}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C107153&amp;Mask=1E9F#Thermo-Condensed</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D4" authorId="0" shapeId="0" xr:uid="{E40BDC6B-934E-411C-B492-C5CD43E5E926}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Hilgeman, Mouroux, Mok, Holan</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E4" authorId="0" shapeId="0" xr:uid="{9BE4DF8B-2AFF-4A6C-9B30-43F0C8BC4258}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Hilgeman, Mouroux, Mok, Holan</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F4" authorId="0" shapeId="0" xr:uid="{22C3A041-08B4-4358-8FFC-0CCF2BF68560}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C288324&amp;Units=SI&amp;Mask=2#Thermo-Condensed</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="0" shapeId="0" xr:uid="{9B46E2A3-89E8-410D-9F36-E3CC4EDF12E7}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C141435&amp;Units=SI&amp;Mask=4#Thermo-Phase</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E5" authorId="0" shapeId="0" xr:uid="{7AFC09FE-6D63-4AB4-9F34-8C6E6346C5F6}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://www.sciencedirect.com/science/article/pii/S1750583613004258</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F5" authorId="0" shapeId="0" xr:uid="{19F57934-8119-42AF-9A95-961B9A767839}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C141435&amp;Units=SI&amp;Mask=2#Thermo-Condensed</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D6" authorId="0" shapeId="0" xr:uid="{A44F0865-2292-4150-8EDA-994F95E330D4}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Ashlee</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E6" authorId="0" shapeId="0" xr:uid="{22EA6CA3-1836-4119-B6E7-99ADB8AE94F6}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Ashlee</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F6" authorId="0" shapeId="0" xr:uid="{7A8F76C3-1C0D-4DE3-9D30-F2E27379947A}">
       <text>
         <r>
           <rPr>
@@ -177,81 +1136,6 @@
           <t xml:space="preserve">
 Source(s):
 1)https://atct.anl.gov/Thermochemical%20Data/version%201.220/species/?species_number=1907</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{849D1544-57C4-43A4-BA3D-7F847C80452D}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Source(s):
-1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C141435&amp;Units=SI&amp;Mask=4#Thermo-Phase</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E3" authorId="0" shapeId="0" xr:uid="{29E8F43A-4689-4EB4-8F76-89740B0C82BA}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Source(s):
-1)https://www.sciencedirect.com/science/article/pii/S1750583613004258</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F3" authorId="0" shapeId="0" xr:uid="{17BF1160-7484-404D-A892-BF5C2E1F290F}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Source(s):
-1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C141435&amp;Units=SI&amp;Mask=2#Thermo-Condensed</t>
         </r>
       </text>
     </comment>
@@ -260,7 +1144,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="34">
   <si>
     <t>Full Name</t>
   </si>
@@ -296,13 +1180,82 @@
   </si>
   <si>
     <t>NCCO</t>
+  </si>
+  <si>
+    <t>Acetamide</t>
+  </si>
+  <si>
+    <t>C2H5NO</t>
+  </si>
+  <si>
+    <t>Imidazole</t>
+  </si>
+  <si>
+    <t>Water</t>
+  </si>
+  <si>
+    <t>H2O</t>
+  </si>
+  <si>
+    <t>O</t>
+  </si>
+  <si>
+    <t>Ethylenediamine</t>
+  </si>
+  <si>
+    <t>CC(N)=O</t>
+  </si>
+  <si>
+    <t>NCCN</t>
+  </si>
+  <si>
+    <t>c1c[nH]cn1</t>
+  </si>
+  <si>
+    <t>Tetrabutylammonium Borohydride</t>
+  </si>
+  <si>
+    <t>[BH4-].CCCC[N+](CCCC)(CCCC)CCCC</t>
+  </si>
+  <si>
+    <t>Ammonia Borane</t>
+  </si>
+  <si>
+    <t>[BH3-][NH3+]</t>
+  </si>
+  <si>
+    <t>Lithium Borohydride</t>
+  </si>
+  <si>
+    <t>[Li+].[BH4-]</t>
+  </si>
+  <si>
+    <t>Sodium Borohydride</t>
+  </si>
+  <si>
+    <t>Glycerol</t>
+  </si>
+  <si>
+    <t>C3H8O3</t>
+  </si>
+  <si>
+    <t>Diglyme</t>
+  </si>
+  <si>
+    <t>C6H14O3</t>
+  </si>
+  <si>
+    <t>Tetraethylammonium Borohydride</t>
+  </si>
+  <si>
+    <t>[B].CC[N+](CC)(CC)CC</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -329,19 +1282,26 @@
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -370,14 +1330,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -712,18 +1672,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3399CF41-2FA5-4790-AC55-DE65A2BCB50A}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -745,44 +1705,242 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2">
+        <v>273.14999999999998</v>
+      </c>
+      <c r="E2">
+        <f>334000*(0.018)</f>
+        <v>6012</v>
+      </c>
+      <c r="F2">
+        <v>-285802</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3">
+        <f>79+273.15</f>
+        <v>352.15</v>
+      </c>
+      <c r="E3">
+        <v>7730</v>
+      </c>
+      <c r="F3">
+        <v>-315890</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B4" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C4" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D4">
         <f>133+273.15</f>
         <v>406.15</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E4">
         <v>10340</v>
       </c>
-      <c r="F2" s="4">
+      <c r="F4">
         <v>-333330</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5">
+        <v>363.7</v>
+      </c>
+      <c r="E5">
+        <v>12500</v>
+      </c>
+      <c r="F5">
+        <v>49800</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6" t="s">
+      <c r="B6" s="5"/>
+      <c r="C6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D6" s="5">
         <v>283.45999999999998</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E6" s="5">
         <v>13800</v>
       </c>
-      <c r="F3" s="6">
+      <c r="F6" s="5">
         <v>-507500</v>
       </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="5">
+        <f>273.15+124</f>
+        <v>397.15</v>
+      </c>
+      <c r="E7" s="5">
+        <v>15800</v>
+      </c>
+      <c r="F7" s="5"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5">
+        <f>(209.1+209.15)/2</f>
+        <v>209.125</v>
+      </c>
+      <c r="E8" s="5">
+        <f>(17.78+17.795)/2*1000</f>
+        <v>17787.5</v>
+      </c>
+      <c r="F8" s="5">
+        <f>(-556.4-569.4)/2*1000</f>
+        <v>-562900</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="6">
+        <f>(292+291+293+291.75)/4</f>
+        <v>291.9375</v>
+      </c>
+      <c r="E9">
+        <f>(18.303+18.285+18.28+18.476)/4*1000</f>
+        <v>18336</v>
+      </c>
+      <c r="F9">
+        <f>(-669.6-668.6)/2</f>
+        <v>-669.1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="5">
+        <v>284.2</v>
+      </c>
+      <c r="E10" s="5">
+        <v>21830</v>
+      </c>
+      <c r="F10" s="5">
+        <v>-63010</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="5">
+        <f>273.15+108</f>
+        <v>381.15</v>
+      </c>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5">
+        <v>-133400</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="5">
+        <f>273.15+268</f>
+        <v>541.15</v>
+      </c>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5">
+        <v>-190800</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5">
+        <v>673.15</v>
+      </c>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F1" xr:uid="{3399CF41-2FA5-4790-AC55-DE65A2BCB50A}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F14">
+      <sortCondition ref="E1"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
@@ -790,10 +1948,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDE786A1-84C7-4241-A3B9-138356725320}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="75" x14ac:dyDescent="0.25">
@@ -818,41 +1981,95 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2">
+        <f>79+273.15</f>
+        <v>352.15</v>
+      </c>
+      <c r="E2">
+        <v>7730</v>
+      </c>
+      <c r="F2">
+        <v>-315890</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3">
+        <v>284.2</v>
+      </c>
+      <c r="E3">
+        <v>21830</v>
+      </c>
+      <c r="F3">
+        <v>-63010</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4">
+        <v>363.7</v>
+      </c>
+      <c r="E4">
+        <v>12500</v>
+      </c>
+      <c r="F4">
+        <v>49800</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5">
+        <v>283.45999999999998</v>
+      </c>
+      <c r="E5">
+        <v>13800</v>
+      </c>
+      <c r="F5">
+        <v>-507500</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B6" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C6" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D6">
         <f>133+273.15</f>
         <v>406.15</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E6">
         <v>10340</v>
       </c>
-      <c r="F2" s="4">
+      <c r="F6">
         <v>-333330</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="6">
-        <v>283.45999999999998</v>
-      </c>
-      <c r="E3" s="6">
-        <v>13800</v>
-      </c>
-      <c r="F3" s="6">
-        <v>-507500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>